<commit_message>
Bo sung kiem thu ADS-B va AMHS
</commit_message>
<xml_diff>
--- a/Pm Số liệu điều hành bay - Mục 1.1.xlsx
+++ b/Pm Số liệu điều hành bay - Mục 1.1.xlsx
@@ -29,7 +29,7 @@
 <file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <cp:lastModifiedBy>NGOQUY</cp:lastModifiedBy>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-04T04:02:27Z</dcterms:modified>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-09-04T04:42:47Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Đạt</t>
   </si>
@@ -132,105 +132,64 @@
     <t>VSD comment</t>
   </si>
   <si>
-    <t>Hợp đồng vi bằng</t>
+    <t>Tự động cập nhật dữ liệu từ email và thư mục lưu trữ</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Thừa phát lại (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>Thừa hành viên</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>)</t>
-    </r>
+    <t>Job hệ thống; Máy chủ thư điện tử; Hệ thống file; Quản trị viên; Người khai thác</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve">1. Truy cập hệ thống theo địa chỉ: </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>https://vibang_hungyen.poc-apps.com</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve">
-2. Đăng nhập bằng tài khoản: vpthads_ta_anhtt, vai trò Thừa hành viên
-3. Chọn menu chức năng: "Vi bằng" -&gt; "Hợp đồng dịch vụ"</t>
-    </r>
+    <t>1. Job định thời kích hoạt quét theo chu kỳ (mặc định 5 phút/lần).
+2. Kết nối hộp thư IMAP/POP3/Exchange và quét thư mục /data/incoming/.
+3. Lấy email chưa đọc/file mới, tải file đính kèm về thư mục tạm.
+4. Kiểm tra phần mở rộng, UTF-8, cấu trúc và kích thước; phân tích theo file mẫu/bảng ánh xạ.
+5. Kiểm tra ràng buộc nghiệp vụ, cập nhật Oracle, lưu bản gốc và ghi audit log.
+6. Di chuyển file theo kết quả xử lý và gửi cảnh báo khi có lỗi.</t>
   </si>
   <si>
-    <t>Thừa phát lại (Thừa hành viên) xem danh sách hợp đồng vi bằng</t>
+    <t>File dữ liệu hợp lệ được chuẩn hóa và cập nhật Oracle trong giao dịch toàn vẹn; bản gốc lưu tại /processed/; audit log đầy đủ; lỗi định dạng vào /error/; vi phạm nghiệp vụ vào /quarantine/ kèm cảnh báo.</t>
   </si>
   <si>
-    <t>Thừa hành viên xem danh sách các hợp đồng dịch vụ trên bảng dữ liệu</t>
+    <t>Quét email và thư mục incoming</t>
   </si>
   <si>
-    <t>Hệ thống hiển thị danh sách các hợp đồng dịch vụ</t>
+    <t>Kích hoạt job; kết nối máy chủ thư điện tử; đọc email chưa đọc và phát hiện file mới trong /data/incoming/.</t>
   </si>
   <si>
-    <t>Thừa phát lại (Thừa hành viên) tìm kiếm trong danh sách hợp đồng vi bằng</t>
+    <t>Hệ thống nhận diện đúng file mới, thông tin tiêu đề/người gửi/thời gian và file đính kèm; không xử lý trùng lặp.</t>
   </si>
   <si>
-    <t>Ở thanh chức năng, Thừa hành viên nhập thông tin về hợp đồng dịch vụ cần tìm kiếm</t>
+    <t>Kiểm tra định dạng và phân tích cú pháp</t>
   </si>
   <si>
-    <t>Hệ thống hiển thị danh sách các hợp đồng dịch vụ theo tiêu chí tìm kiếm</t>
+    <t>Nạp file CSV/XLSX/XML/JSON; kiểm tra phần mở rộng, mã UTF-8, cấu trúc, kích thước; đối chiếu file mẫu và bảng ánh xạ; kiểm tra ràng buộc nghiệp vụ.</t>
   </si>
   <si>
-    <t>Thừa phát lại (Thừa hành viên) thêm mới hợp đồng vi bằng</t>
+    <t>File hợp lệ được chuẩn hóa; file sai định dạng chuyển /error/ kèm .log WARNING; file vi phạm ràng buộc bị hủy giao dịch và chuyển /quarantine/.</t>
   </si>
   <si>
-    <t>1. Ở thanh chức năng, Thừa hành viên chọn nút "Thêm mới"
-2. Nhập thông tin hợp đồng dịch vụ
-3. Chọn nút "Lưu"</t>
+    <t>Cập nhật cơ sở dữ liệu và lưu trữ bản gốc</t>
   </si>
   <si>
-    <t>Hệ thống thêm mới thành công hợp đồng dịch vụ, có thông báo thêm mới thành công</t>
+    <t>Ghi dữ liệu đã chuẩn hóa vào Oracle; lưu file gốc; ghi nhật ký kiểm toán; đánh dấu email đã đọc.</t>
   </si>
   <si>
-    <t>Thừa phát lại (Thừa hành viên) xem hợp đồng vi bằng</t>
+    <t>Dữ liệu cập nhật thành công với toàn vẹn giao dịch; file có tên chuẩn tại /processed/; audit log lưu tối thiểu 5 năm; gửi thông báo hoàn thành.</t>
   </si>
   <si>
-    <t>Trong danh sách hợp đồng dịch vụ, cột "Thao tác", Thừa hành viên chọn biểu tượng "Xem" hợp đồng dịch vụ</t>
+    <t>Xử lý ngoại lệ và cảnh báo</t>
   </si>
   <si>
-    <t>Hệ thống hiển thị thông tin hợp đồng dịch vụ</t>
+    <t>Mô phỏng file trùng, mất kết nối Oracle, máy chủ email không khả dụng và email không có file đính kèm.</t>
+  </si>
+  <si>
+    <t>File trùng được bỏ qua và ghi log; lỗi DB thử lại tối đa 3 lần rồi cảnh báo CRITICAL; lỗi máy chủ email bỏ qua chu kỳ và cảnh báo sau 3 lần; email không đính kèm được ghi log.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -288,10 +247,6 @@
       <u/>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <name val="Times New Roman"/>
     </font>
   </fonts>
@@ -409,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -472,6 +427,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -692,7 +650,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell 3567\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026\QLB\TrienKhai\ATFM_WEB\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -866,7 +824,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -924,35 +882,22 @@
       </c>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="66" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>1</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Tự động cập nhật dữ liệu từ email và thư mục lưu trữ</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>Job hệ thống; Máy chủ thư điện tử; Hệ thống file; Quản trị viên; Người khai thác</t>
-        </is>
+      <c r="B6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>23</v>
       </c>
       <c r="D6" s="12"/>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>1. Job định thời kích hoạt quét theo chu kỳ (mặc định 5 phút/lần).
-2. Kết nối hộp thư IMAP/POP3/Exchange và quét thư mục /data/incoming/.
-3. Lấy email chưa đọc/file mới, tải file đính kèm về thư mục tạm.
-4. Kiểm tra phần mở rộng, UTF-8, cấu trúc và kích thước; phân tích theo file mẫu/bảng ánh xạ.
-5. Kiểm tra ràng buộc nghiệp vụ, cập nhật Oracle, lưu bản gốc và ghi audit log.
-6. Di chuyển file theo kết quả xử lý và gửi cảnh báo khi có lỗi.</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>File dữ liệu hợp lệ được chuẩn hóa và cập nhật Oracle trong giao dịch toàn vẹn; bản gốc lưu tại /processed/; audit log đầy đủ; lỗi định dạng vào /error/; vi phạm nghiệp vụ vào /quarantine/ kèm cảnh báo.</t>
-        </is>
+      <c r="E6" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>25</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="2"/>
@@ -970,20 +915,14 @@
       <c r="A7" s="14"/>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>Quét email và thư mục incoming</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="inlineStr">
-        <is>
-          <t>Kích hoạt job; kết nối máy chủ thư điện tử; đọc email chưa đọc và phát hiện file mới trong /data/incoming/.</t>
-        </is>
-      </c>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>Hệ thống nhận diện đúng file mới, thông tin tiêu đề/người gửi/thời gian và file đính kèm; không xử lý trùng lặp.</t>
-        </is>
+      <c r="D7" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>28</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="5"/>
@@ -1001,20 +940,14 @@
       <c r="A8" s="14"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>Kiểm tra định dạng và phân tích cú pháp</t>
-        </is>
-      </c>
-      <c r="E8" s="15" t="inlineStr">
-        <is>
-          <t>Nạp file CSV/XLSX/XML/JSON; kiểm tra phần mở rộng, mã UTF-8, cấu trúc, kích thước; đối chiếu file mẫu và bảng ánh xạ; kiểm tra ràng buộc nghiệp vụ.</t>
-        </is>
-      </c>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
-          <t>File hợp lệ được chuẩn hóa; file sai định dạng chuyển /error/ kèm .log WARNING; file vi phạm ràng buộc bị hủy giao dịch và chuyển /quarantine/.</t>
-        </is>
+      <c r="D8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>31</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="5"/>
@@ -1032,20 +965,14 @@
       <c r="A9" s="14"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Cập nhật cơ sở dữ liệu và lưu trữ bản gốc</t>
-        </is>
-      </c>
-      <c r="E9" s="15" t="inlineStr">
-        <is>
-          <t>Ghi dữ liệu đã chuẩn hóa vào Oracle; lưu file gốc; ghi nhật ký kiểm toán; đánh dấu email đã đọc.</t>
-        </is>
-      </c>
-      <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>Dữ liệu cập nhật thành công với toàn vẹn giao dịch; file có tên chuẩn tại /processed/; audit log lưu tối thiểu 5 năm; gửi thông báo hoàn thành.</t>
-        </is>
+      <c r="D9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="5"/>
@@ -1063,20 +990,14 @@
       <c r="A10" s="14"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>Xử lý ngoại lệ và cảnh báo</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>Mô phỏng file trùng, mất kết nối Oracle, máy chủ email không khả dụng và email không có file đính kèm.</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>File trùng được bỏ qua và ghi log; lỗi DB thử lại tối đa 3 lần rồi cảnh báo CRITICAL; lỗi máy chủ email bỏ qua chu kỳ và cảnh báo sau 3 lần; email không đính kèm được ghi log.</t>
-        </is>
+      <c r="D10" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="5"/>
@@ -1091,12 +1012,35 @@
       <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Thu thập và xử lý dữ liệu ADS-B cho khai thác O/F</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Cổng ADS-B; Người khai thác ATFM; Job hệ thống; Quản trị viên</t>
+        </is>
+      </c>
       <c r="D11" s="11"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>1. Kết nối cổng ADS-B Gateway và nhận bản tin vị trí theo thời gian thực.
+2. Phân tích, chuẩn hóa và lọc nhiễu bản tin.
+3. Đối chiếu với FPL theo khóa tổng hợp; xác định trạng thái ENTRY/IN-FIR/EXIT trong FIR Hà Nội và Hồ Chí Minh.
+4. Cập nhật trạng thái O/F, lưu trajectory, hiển thị bản đồ/bảng điều khiển và ghi log sự kiện.</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Dữ liệu O/F cập nhật thời gian thực với độ trễ ≤ 3 giây; trajectory được lưu; chuyến bay không đối chiếu được gắn UNKNOWN_FLIGHT và cảnh báo NOPERM; ghi đủ ENTRY/EXIT.</t>
+        </is>
+      </c>
       <c r="G11" s="7"/>
       <c r="H11" s="5"/>
       <c r="I11" s="7"/>
@@ -1113,9 +1057,21 @@
       <c r="A12" s="14"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Tiếp nhận và phân tích bản tin ADS-B</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Kết nối Gateway; nhận bản tin mỗi 1-2 giây; kiểm tra cấu trúc, chuẩn hóa dữ liệu và lọc bản tin nhiễu.</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Bản tin hợp lệ được xử lý liên tục; dữ liệu sai/ngoài FIR bị loại và ghi log; không làm gián đoạn luồng.</t>
+        </is>
+      </c>
       <c r="G12" s="7"/>
       <c r="H12" s="5"/>
       <c r="I12" s="7"/>
@@ -1132,9 +1088,21 @@
       <c r="A13" s="14"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Đối chiếu ADS-B với kế hoạch bay FPL</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Dùng khóa callsign + dep_icao + arr_icao + flight_date để đối chiếu bản tin với FPL.</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>Đối chiếu một-một đúng bản tin/FPL; chuyến bay không khớp được gắn UNKNOWN_FLIGHT và phát cảnh báo NOPERM.</t>
+        </is>
+      </c>
       <c r="G13" s="7"/>
       <c r="H13" s="5"/>
       <c r="I13" s="7"/>
@@ -1151,9 +1119,21 @@
       <c r="A14" s="14"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Cập nhật trạng thái O/F và trajectory</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Xác định ENTRY/IN-FIR/EXIT; cập nhật trạng thái theo thời gian thực; lưu đường bay vào flight_trajectory; hiển thị bản đồ và dashboard.</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Trạng thái cập nhật đúng, độ trễ ≤ 3 giây; trajectory lưu tối thiểu 2 năm; log đầy đủ sự kiện ENTRY/EXIT.</t>
+        </is>
+      </c>
       <c r="G14" s="7"/>
       <c r="H14" s="5"/>
       <c r="I14" s="7"/>
@@ -1170,9 +1150,21 @@
       <c r="A15" s="14"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Xử lý mất kết nối, mất tín hiệu và xung đột</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Mô phỏng mất Gateway, gián đoạn đường bay &gt;30 giây, trùng callsign và dữ liệu ngoài FIR Việt Nam.</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Tự động nối lại có backoff và banner; gắn TRACK_LOST/giữ vị trí cuối; ưu tiên FPL nộp gần nhất; dữ liệu ngoài FIR bị loại và ghi thống kê.</t>
+        </is>
+      </c>
       <c r="G15" s="7"/>
       <c r="H15" s="5"/>
       <c r="I15" s="15"/>
@@ -1186,12 +1178,35 @@
       <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Kết nối trực tiếp AMHS để gửi/nhận điện văn</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Cổng AMHS; Quản trị viên; Người khai thác</t>
+        </is>
+      </c>
       <c r="D16" s="12"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="7"/>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>1. Kết nối trực tiếp cơ sở dữ liệu AMHS qua Gateway.
+2. Luồng inbound truy vấn điện văn mới, phân tích AFTN theo ICAO và cập nhật trạng thái chuyến bay.
+3. Luồng outbound chọn chuyến bay/loại điện văn, sinh theo mẫu ICAO, kiểm tra cú pháp và đẩy sang AMHS.
+4. Ghi audit log, xác nhận gửi và xử lý lỗi/quarantine.</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Điện văn đến cập nhật trạng thái ≤ 5 giây; điện văn đi đúng chuẩn ICAO và có xác nhận; toàn bộ điện văn/audit log được lưu; lỗi vào /quarantine/ và cảnh báo.</t>
+        </is>
+      </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
@@ -1208,9 +1223,21 @@
       <c r="A17" s="14"/>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Nhận và phân tích điện văn AMHS (inbound)</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Job truy vấn AMHS mỗi 1-5 giây; lấy lô điện văn FPL/DEP/ARR/CHG/CNL/DLA; phân tích cú pháp ICAO và trích xuất dữ liệu.</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Điện văn hợp lệ được xác thực, cập nhật trạng thái chuyến bay trong ≤ 5 giây; message_id, loại, callsign, hướng, thời gian được ghi log.</t>
+        </is>
+      </c>
       <c r="G17" s="7"/>
       <c r="H17" s="5"/>
       <c r="I17" s="7"/>
@@ -1227,9 +1254,21 @@
       <c r="A18" s="14"/>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Sinh và gửi điện văn AMHS (outbound)</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Người khai thác chọn chuyến bay và loại điện văn; hệ thống tự điền dữ liệu theo template ICAO, kiểm tra cú pháp rồi ghi vào AMHS.</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Điện văn đúng Doc 4444/4445, gửi thành công kèm xác nhận; trạng thái và audit log được cập nhật.</t>
+        </is>
+      </c>
       <c r="G18" s="7"/>
       <c r="H18" s="5"/>
       <c r="I18" s="7"/>
@@ -1246,9 +1285,21 @@
       <c r="A19" s="14"/>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Bảo mật, lưu trữ và kiểm soát tải</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra TLS 1.3/X.509, mã hóa AES-256 khi lưu, quyền ADMIN_AMHS_CONFIG và tải 5.000 bản tin/giờ (đỉnh 10.000).</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Kết nối bảo mật, người không đủ quyền bị từ chối; dữ liệu lưu tối thiểu 60 ngày; hệ thống đáp ứng thông lượng yêu cầu.</t>
+        </is>
+      </c>
       <c r="G19" s="7"/>
       <c r="H19" s="5"/>
       <c r="I19" s="7"/>
@@ -1265,9 +1316,21 @@
       <c r="A20" s="14"/>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Xử lý mất kết nối, sai cú pháp và trùng điện văn</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Mô phỏng mất AMHS, điện văn sai ICAO, chứng chỉ hết hạn, điện văn trùng và AMHS quá tải.</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Xếp hàng và tự kết nối lại; sai cú pháp chuyển /quarantine/ và cảnh báo; cảnh báo chứng chỉ trước 30 ngày; trùng trong 24 giờ bỏ qua; giới hạn tốc độ theo hàng đợi ưu tiên.</t>
+        </is>
+      </c>
       <c r="G20" s="7"/>
       <c r="H20" s="5"/>
       <c r="I20" s="7"/>

</xml_diff>